<commit_message>
Refresh price registry workbooks
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments/pricing/input/price_registry_elena_2026-07-28.xlsx
+++ b/experiments/pricing/input/price_registry_elena_2026-07-28.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Прайс по видам работ" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Бетон + песок" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Пиломатериалы (Олег)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Блокпаротермшидель (Алексей)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Металл (Алексей)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Утеплителипленкимастика (Олег)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прайс по видам работ" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Бетон + песок" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Пиломатериалы (Олег)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Блокпаротермшидель (Алексей)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Металл (Алексей)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Утеплителипленкимастика (Олег)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -549,7 +549,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>8</col>
@@ -564,17 +564,17 @@
         <cNvPicPr preferRelativeResize="0"/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -2741,10 +2741,22 @@
     </row>
     <row r="47">
       <c r="A47" s="53" t="n"/>
-      <c r="B47" s="53" t="n"/>
-      <c r="C47" s="53" t="n"/>
-      <c r="D47" s="53" t="n"/>
-      <c r="E47" s="61" t="n"/>
+      <c r="B47" s="53" t="inlineStr">
+        <is>
+          <t>Укладка ЦСП в 2 слоя (24мм)</t>
+        </is>
+      </c>
+      <c r="C47" s="53" t="inlineStr">
+        <is>
+          <t>м2</t>
+        </is>
+      </c>
+      <c r="D47" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="61" t="n">
+        <v>900</v>
+      </c>
       <c r="F47" s="53" t="n"/>
       <c r="G47" s="53" t="n"/>
       <c r="H47" s="53" t="n"/>
@@ -33591,7 +33603,7 @@
         </is>
       </c>
       <c r="C23" s="63" t="n">
-        <v>59.55</v>
+        <v>66.31999999999999</v>
       </c>
     </row>
     <row r="24">
@@ -33666,7 +33678,7 @@
         </is>
       </c>
       <c r="C28" s="63" t="n">
-        <v>1146.91</v>
+        <v>1166.23</v>
       </c>
     </row>
     <row r="29">
@@ -33681,7 +33693,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>1146.91</v>
+        <v>1166.23</v>
       </c>
     </row>
     <row r="30">
@@ -33739,7 +33751,19 @@
       <c r="C33" s="63" t="n"/>
     </row>
     <row r="34">
-      <c r="C34" s="64" t="n"/>
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>Цементно-стружечная плита (ЦСП I) толщина 12 мм 3200х1200</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="C34" s="64" t="n">
+        <v>2388</v>
+      </c>
     </row>
     <row r="35">
       <c r="C35" s="64" t="n"/>

</xml_diff>